<commit_message>
Update D&R pricing with confirmed terms: tack minimum, standby hourly, flat prime
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W6veyHJxmKEQ2ybPTx8WzX
</commit_message>
<xml_diff>
--- a/pricing/DR_Prime_Tack_Pricing.xlsx
+++ b/pricing/DR_Prime_Tack_Pricing.xlsx
@@ -35,7 +35,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Hours are an estimator assumption, not from D&amp;R. Include drive time if they bill portal-to-portal.</t>
+          <t xml:space="preserve">Only if D&amp;R's truck stays on site all day (e.g. community jobs). Billed from their yard and back, so include drive time. Hours are the estimator's call, not a D&amp;R number.</t>
         </r>
       </text>
     </comment>
@@ -57,7 +57,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Assumption, not from D&amp;R. Change to suit the job.</t>
+          <t xml:space="preserve">Assumption, not from D&amp;R: ~8 hrs on site + ~2 hrs yard-to-yard travel. Change to suit the job.</t>
         </r>
       </text>
     </comment>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
   <si>
     <t xml:space="preserve">D&amp;R Prime and Tack — Vendor Rate Sheet (Paramount Asphalt)</t>
   </si>
@@ -104,13 +104,13 @@
     <t xml:space="preserve">Quoted by D&amp;R (= 0.10 gal/SY)</t>
   </si>
   <si>
-    <t xml:space="preserve">Tack — truck/crew hourly</t>
+    <t xml:space="preserve">Tack — standby hourly (optional)</t>
   </si>
   <si>
     <t xml:space="preserve">$/hr</t>
   </si>
   <si>
-    <t xml:space="preserve">Quoted by D&amp;R. Confirm portal-to-portal vs. on-site only</t>
+    <t xml:space="preserve">On top of $/gal. Only if truck stays on site all day (e.g. community jobs). Billed yard-to-yard</t>
   </si>
   <si>
     <t xml:space="preserve">Prime</t>
@@ -119,33 +119,42 @@
     <t xml:space="preserve">$/SY</t>
   </si>
   <si>
+    <t xml:space="preserve">Flat rate, primes whole job. No hourly</t>
+  </si>
+  <si>
     <t xml:space="preserve">Prime &amp; sand</t>
   </si>
   <si>
-    <t xml:space="preserve">Minimum (prime / prime &amp; sand)</t>
+    <t xml:space="preserve">Minimum — tack, prime, prime &amp; sand</t>
   </si>
   <si>
     <t xml:space="preserve">SY</t>
   </si>
   <si>
-    <t xml:space="preserve">Quoted by D&amp;R. Confirm whether it also applies to tack</t>
+    <t xml:space="preserve">Applies to all three services</t>
   </si>
   <si>
     <t xml:space="preserve">Derived</t>
   </si>
   <si>
+    <t xml:space="preserve">Tack — minimum charge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,500 SY ÷ 10 SY/gal × $/gal (no standby)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tack — material cost per SY</t>
   </si>
   <si>
-    <t xml:space="preserve">Excludes hourly truck time</t>
+    <t xml:space="preserve">Excludes standby hours</t>
   </si>
   <si>
     <t xml:space="preserve">Prime — minimum charge</t>
   </si>
   <si>
-    <t xml:space="preserve">$</t>
-  </si>
-  <si>
     <t xml:space="preserve">1,500 SY × prime rate</t>
   </si>
   <si>
@@ -155,22 +164,13 @@
     <t xml:space="preserve">1,500 SY × prime &amp; sand rate</t>
   </si>
   <si>
-    <t xml:space="preserve">Open questions to confirm with D&amp;R before relying on these numbers:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Is the $110/hr charged on top of the $5.75/gal for tack, or is it a separate minimum/mobilization?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Does the 1,500 SY minimum apply to tack, or only prime / prime &amp; sand?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Do the prime rates ($0.50 / $0.70 per SY) include labor, truck and sand, or is hourly added?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Is hourly billed portal-to-portal (from their yard) or on-site time only? Any trip/mobilization charge?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Is 10 SY/gal their standard application rate, or adjustable per spec (e.g., 0.05 gal/SY)?</t>
+    <t xml:space="preserve">Still open with D&amp;R:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Is 10 SY/gal (0.10 gal/SY) their standard tack rate, or will they shoot a lighter spec (e.g. 0.05 gal/SY)?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Is the tack minimum billed as 150 gal ($862.50) even if fewer gallons go down?</t>
   </si>
   <si>
     <t xml:space="preserve">D&amp;R Prime &amp; Tack — Job Estimator</t>
@@ -185,10 +185,16 @@
     <t xml:space="preserve">Square yards</t>
   </si>
   <si>
-    <t xml:space="preserve">Example values — overwrite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated truck hours</t>
+    <t xml:space="preserve">Example value — overwrite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standby hours (yard-to-yard)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 unless he stays all day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Billable SY (1,500 min)</t>
   </si>
   <si>
     <t xml:space="preserve">Gallons</t>
@@ -197,7 +203,7 @@
     <t xml:space="preserve">Material</t>
   </si>
   <si>
-    <t xml:space="preserve">Hourly</t>
+    <t xml:space="preserve">Standby hourly</t>
   </si>
   <si>
     <t xml:space="preserve">Tack total</t>
@@ -209,9 +215,6 @@
     <t xml:space="preserve">PRIME</t>
   </si>
   <si>
-    <t xml:space="preserve">Billable SY (1,500 min)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Prime total</t>
   </si>
   <si>
@@ -230,10 +233,10 @@
     <t xml:space="preserve">D&amp;R Cost Quick Reference by Job Size</t>
   </si>
   <si>
-    <t xml:space="preserve">Tack shown as material only + with an hourly allowance. Prime columns have the 1,500 SY minimum applied.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tack hrs allowance:</t>
+    <t xml:space="preserve">1,500 SY minimum applied to every column. 'Tack + Full Day' adds standby hours (yard-to-yard) at $110/hr.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full-day standby hrs:</t>
   </si>
   <si>
     <t xml:space="preserve">Square Yards</t>
@@ -242,10 +245,10 @@
     <t xml:space="preserve">Tack Gallons</t>
   </si>
   <si>
-    <t xml:space="preserve">Tack Material</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tack + Hourly</t>
+    <t xml:space="preserve">Tack (no standby)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tack + Full Day</t>
   </si>
   <si>
     <t xml:space="preserve">Prime &amp; Sand</t>
@@ -486,15 +489,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -778,7 +781,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
@@ -867,12 +870,12 @@
         <v>16</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>0.7</v>
@@ -881,100 +884,100 @@
         <v>16</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B10" s="6" t="n">
         <v>1500</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B13" s="8" t="n">
+        <f aca="false">B10/B6*B5</f>
+        <v>862.5</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="8" t="n">
         <f aca="false">B5/B6</f>
         <v>0.575</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="9" t="n">
+      <c r="D14" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="9" t="n">
         <f aca="false">B10*B8</f>
         <v>750</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="9" t="n">
+      <c r="C15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="9" t="n">
         <f aca="false">B10*B9</f>
         <v>1050</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>29</v>
+      <c r="C16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
-        <v>30</v>
+      <c r="A18" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1040,57 +1043,69 @@
         <v>40</v>
       </c>
       <c r="B6" s="14" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B7" s="15" t="n">
-        <f aca="false">B5/Rates!$B$6</f>
-        <v>300</v>
+        <f aca="false">IF(B5&gt;0,MAX(B5,Rates!$B$10),0)</f>
+        <v>3000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" s="8" t="n">
-        <f aca="false">B7*Rates!$B$5</f>
-        <v>1725</v>
+        <v>43</v>
+      </c>
+      <c r="B8" s="16" t="n">
+        <f aca="false">B7/Rates!$B$6</f>
+        <v>300</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B9" s="8" t="n">
+        <f aca="false">B8*Rates!$B$5</f>
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="8" t="n">
         <f aca="false">B6*Rates!$B$7</f>
-        <v>330</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="16" t="n">
-        <f aca="false">B8+B9</f>
-        <v>2055</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="8" t="n">
-        <f aca="false">IF(B5&gt;0,B10/B5,0)</f>
-        <v>0.685</v>
+      <c r="A11" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="17" t="n">
+        <f aca="false">B9+B10</f>
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="8" t="n">
+        <f aca="false">IF(B5&gt;0,B11/B5,0)</f>
+        <v>0.575</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -1105,25 +1120,25 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="B15" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="B15" s="15" t="n">
         <f aca="false">IF(B14&gt;0,MAX(B14,Rates!$B$10),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="B16" s="17" t="n">
         <f aca="false">B15*Rates!$B$8</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">IF(B14&gt;0,B16/B14,0)</f>
@@ -1132,7 +1147,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
@@ -1147,25 +1162,25 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="B21" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="B21" s="15" t="n">
         <f aca="false">IF(B20&gt;0,MAX(B20,Rates!$B$10),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="B22" s="16" t="n">
+        <v>51</v>
+      </c>
+      <c r="B22" s="17" t="n">
         <f aca="false">B21*Rates!$B$9</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">IF(B20&gt;0,B22/B20,0)</f>
@@ -1174,16 +1189,16 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B25" s="19" t="n">
-        <f aca="false">B10+B16+B22</f>
-        <v>2055</v>
+        <f aca="false">B11+B16+B22</f>
+        <v>1725</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1214,7 +1229,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1224,35 +1239,35 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E3" s="21" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F3" s="22" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>15</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1260,16 +1275,16 @@
         <v>500</v>
       </c>
       <c r="B6" s="24" t="n">
-        <f aca="false">A6/Rates!$B$6</f>
-        <v>50</v>
+        <f aca="false">MAX(A6,Rates!$B$10)/Rates!$B$6</f>
+        <v>150</v>
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">B6*Rates!$B$5</f>
-        <v>287.5</v>
+        <v>862.5</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">C6+$F$3*Rates!$B$7</f>
-        <v>617.5</v>
+        <v>1962.5</v>
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">MAX(A6,Rates!$B$10)*Rates!$B$8</f>
@@ -1285,16 +1300,16 @@
         <v>1000</v>
       </c>
       <c r="B7" s="24" t="n">
-        <f aca="false">A7/Rates!$B$6</f>
-        <v>100</v>
+        <f aca="false">MAX(A7,Rates!$B$10)/Rates!$B$6</f>
+        <v>150</v>
       </c>
       <c r="C7" s="9" t="n">
         <f aca="false">B7*Rates!$B$5</f>
-        <v>575</v>
+        <v>862.5</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">C7+$F$3*Rates!$B$7</f>
-        <v>905</v>
+        <v>1962.5</v>
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">MAX(A7,Rates!$B$10)*Rates!$B$8</f>
@@ -1310,7 +1325,7 @@
         <v>1500</v>
       </c>
       <c r="B8" s="24" t="n">
-        <f aca="false">A8/Rates!$B$6</f>
+        <f aca="false">MAX(A8,Rates!$B$10)/Rates!$B$6</f>
         <v>150</v>
       </c>
       <c r="C8" s="9" t="n">
@@ -1319,7 +1334,7 @@
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">C8+$F$3*Rates!$B$7</f>
-        <v>1192.5</v>
+        <v>1962.5</v>
       </c>
       <c r="E8" s="9" t="n">
         <f aca="false">MAX(A8,Rates!$B$10)*Rates!$B$8</f>
@@ -1335,7 +1350,7 @@
         <v>2000</v>
       </c>
       <c r="B9" s="24" t="n">
-        <f aca="false">A9/Rates!$B$6</f>
+        <f aca="false">MAX(A9,Rates!$B$10)/Rates!$B$6</f>
         <v>200</v>
       </c>
       <c r="C9" s="9" t="n">
@@ -1344,7 +1359,7 @@
       </c>
       <c r="D9" s="9" t="n">
         <f aca="false">C9+$F$3*Rates!$B$7</f>
-        <v>1480</v>
+        <v>2250</v>
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">MAX(A9,Rates!$B$10)*Rates!$B$8</f>
@@ -1360,7 +1375,7 @@
         <v>2500</v>
       </c>
       <c r="B10" s="24" t="n">
-        <f aca="false">A10/Rates!$B$6</f>
+        <f aca="false">MAX(A10,Rates!$B$10)/Rates!$B$6</f>
         <v>250</v>
       </c>
       <c r="C10" s="9" t="n">
@@ -1369,7 +1384,7 @@
       </c>
       <c r="D10" s="9" t="n">
         <f aca="false">C10+$F$3*Rates!$B$7</f>
-        <v>1767.5</v>
+        <v>2537.5</v>
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">MAX(A10,Rates!$B$10)*Rates!$B$8</f>
@@ -1385,7 +1400,7 @@
         <v>3000</v>
       </c>
       <c r="B11" s="24" t="n">
-        <f aca="false">A11/Rates!$B$6</f>
+        <f aca="false">MAX(A11,Rates!$B$10)/Rates!$B$6</f>
         <v>300</v>
       </c>
       <c r="C11" s="9" t="n">
@@ -1394,7 +1409,7 @@
       </c>
       <c r="D11" s="9" t="n">
         <f aca="false">C11+$F$3*Rates!$B$7</f>
-        <v>2055</v>
+        <v>2825</v>
       </c>
       <c r="E11" s="9" t="n">
         <f aca="false">MAX(A11,Rates!$B$10)*Rates!$B$8</f>
@@ -1410,7 +1425,7 @@
         <v>4000</v>
       </c>
       <c r="B12" s="24" t="n">
-        <f aca="false">A12/Rates!$B$6</f>
+        <f aca="false">MAX(A12,Rates!$B$10)/Rates!$B$6</f>
         <v>400</v>
       </c>
       <c r="C12" s="9" t="n">
@@ -1419,7 +1434,7 @@
       </c>
       <c r="D12" s="9" t="n">
         <f aca="false">C12+$F$3*Rates!$B$7</f>
-        <v>2630</v>
+        <v>3400</v>
       </c>
       <c r="E12" s="9" t="n">
         <f aca="false">MAX(A12,Rates!$B$10)*Rates!$B$8</f>
@@ -1435,7 +1450,7 @@
         <v>5000</v>
       </c>
       <c r="B13" s="24" t="n">
-        <f aca="false">A13/Rates!$B$6</f>
+        <f aca="false">MAX(A13,Rates!$B$10)/Rates!$B$6</f>
         <v>500</v>
       </c>
       <c r="C13" s="9" t="n">
@@ -1444,7 +1459,7 @@
       </c>
       <c r="D13" s="9" t="n">
         <f aca="false">C13+$F$3*Rates!$B$7</f>
-        <v>3205</v>
+        <v>3975</v>
       </c>
       <c r="E13" s="9" t="n">
         <f aca="false">MAX(A13,Rates!$B$10)*Rates!$B$8</f>
@@ -1460,7 +1475,7 @@
         <v>7500</v>
       </c>
       <c r="B14" s="24" t="n">
-        <f aca="false">A14/Rates!$B$6</f>
+        <f aca="false">MAX(A14,Rates!$B$10)/Rates!$B$6</f>
         <v>750</v>
       </c>
       <c r="C14" s="9" t="n">
@@ -1469,7 +1484,7 @@
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">C14+$F$3*Rates!$B$7</f>
-        <v>4642.5</v>
+        <v>5412.5</v>
       </c>
       <c r="E14" s="9" t="n">
         <f aca="false">MAX(A14,Rates!$B$10)*Rates!$B$8</f>
@@ -1485,7 +1500,7 @@
         <v>10000</v>
       </c>
       <c r="B15" s="24" t="n">
-        <f aca="false">A15/Rates!$B$6</f>
+        <f aca="false">MAX(A15,Rates!$B$10)/Rates!$B$6</f>
         <v>1000</v>
       </c>
       <c r="C15" s="9" t="n">
@@ -1494,7 +1509,7 @@
       </c>
       <c r="D15" s="9" t="n">
         <f aca="false">C15+$F$3*Rates!$B$7</f>
-        <v>6080</v>
+        <v>6850</v>
       </c>
       <c r="E15" s="9" t="n">
         <f aca="false">MAX(A15,Rates!$B$10)*Rates!$B$8</f>
@@ -1510,7 +1525,7 @@
         <v>15000</v>
       </c>
       <c r="B16" s="24" t="n">
-        <f aca="false">A16/Rates!$B$6</f>
+        <f aca="false">MAX(A16,Rates!$B$10)/Rates!$B$6</f>
         <v>1500</v>
       </c>
       <c r="C16" s="9" t="n">
@@ -1519,7 +1534,7 @@
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">C16+$F$3*Rates!$B$7</f>
-        <v>8955</v>
+        <v>9725</v>
       </c>
       <c r="E16" s="9" t="n">
         <f aca="false">MAX(A16,Rates!$B$10)*Rates!$B$8</f>
@@ -1535,7 +1550,7 @@
         <v>20000</v>
       </c>
       <c r="B17" s="24" t="n">
-        <f aca="false">A17/Rates!$B$6</f>
+        <f aca="false">MAX(A17,Rates!$B$10)/Rates!$B$6</f>
         <v>2000</v>
       </c>
       <c r="C17" s="9" t="n">
@@ -1544,7 +1559,7 @@
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">C17+$F$3*Rates!$B$7</f>
-        <v>11830</v>
+        <v>12600</v>
       </c>
       <c r="E17" s="9" t="n">
         <f aca="false">MAX(A17,Rates!$B$10)*Rates!$B$8</f>

</xml_diff>